<commit_message>
refactor: rebrand the estimation kit to RB
- org, images and CI under foundryRB (ghcr.io/foundryrb, foundryRB/rb-ci)
- hosts on rb-foundry.com
- appearance shell, docs theme and lockups in the RB identity: the RB tile,
  no flag, green accent, system fonts
- remove the previous brand's fonts and logos
- replace the demo-acme project with an invented field-service example in the current data layout
- quoter and financial model workbook templates in the RB identity; default brand colour #00A86B
</commit_message>
<xml_diff>
--- a/engine/adapters/outbound/excel/templates/Financial Model Template.xlsx
+++ b/engine/adapters/outbound/excel/templates/Financial Model Template.xlsx
@@ -121,13 +121,13 @@
     <t>Customer Pays</t>
   </si>
   <si>
-    <t>Celfocus Profit (Margin)</t>
+    <t>RB Profit (Margin)</t>
   </si>
   <si>
     <t>Customer Funded Cost</t>
   </si>
   <si>
-    <t>Celfocus Cost Contribution</t>
+    <t>RB Cost Contribution</t>
   </si>
   <si>
     <t>S1) Full Customer Funding</t>

</xml_diff>